<commit_message>
docs: 화면 목록 순서 W01~W24, A01~A05
</commit_message>
<xml_diff>
--- a/docs/요구사항_정의서_파이온.xlsx
+++ b/docs/요구사항_정의서_파이온.xlsx
@@ -18755,864 +18755,864 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>A01</t>
+          <t>W01</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>관리자 · 미션 · 가입자 · 통계 · 열람 기록</t>
+          <t>서비스 소개 · 시작하기</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>미션 노출 → 가입자 → 통계 → 열람 기록</t>
+          <t>소개 → 시작하기</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>왼쪽 메뉴(11개), 표, 필터, 검색</t>
+          <t>서비스 한 줄 소개, 핵심 기능 3단계 안내, 시작하기 CTA</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>REQ-ADM-001, REQ-ADM-002, REQ-ADM-003, REQ-ADM-004, REQ-ADM-012</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>A02</t>
+          <t>W02</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>관리자 · 문의 · 비회원 문의</t>
+          <t>회원가입 · 로그인 · 동의</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>목록 → 열어서 답변</t>
+          <t>계정 생성 → 필수 동의</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>상태 필터, 문의 목록, 답변 입력</t>
+          <t>가입 폼, 로그인 폼, 비밀번호 재설정, 약관·건강정보 동의 체크</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>REQ-ADM-005, REQ-ADM-006, REQ-INQ-002, REQ-INQ-003</t>
+          <t>REQ-USER-001, REQ-USER-002, REQ-USER-004, REQ-CONSENT-001, REQ-CONSENT-003, NFR-SEC-003, NFR-SEC-006</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>A03</t>
+          <t>W03</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>관리자 · 공지 · 신고 · 글 관리</t>
+          <t>이용 적합성 · 응급 확인</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>공지 올리기 / 신고 처리 / 글 숨김·삭제</t>
+          <t>안전 문진 → 서비스 분기</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>공지 폼, 신고 표, 글 표, 계정 정지·삭제</t>
+          <t>긴급 증상 문진, 119 전화 버튼, 연령·기진단 확인, 부적합 사유 안내</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>REQ-ADM-007, REQ-ADM-008, REQ-ADM-009, REQ-ADM-013, REQ-NOTICE-001, REQ-COMM-008</t>
+          <t>REQ-ELIG-001, REQ-ELIG-002, REQ-ELIG-003, REQ-ELIG-004, NFR-SAFE-004</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>A04</t>
+          <t>W04</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>관리자 · 공통 챌린지 · 테스트 계정 삭제</t>
+          <t>건강정보 입력</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>공통 챌린지 열기·확정 / 테스트 계정 삭제</t>
+          <t>직접 입력 → 검증</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>챌린지 폼·카드, 순위 확정, 미리보기·삭제</t>
+          <t>기본 정보, 계측·혈압, 가족력, 검진 결과지 사진 채우기, 필드 오류 표시, 검진 이력 추가</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>REQ-ADM-010, REQ-ADM-011, REQ-CCHAL-005</t>
+          <t>REQ-HEALTH-001, REQ-HEALTH-002, REQ-HEALTH-003, REQ-HEALTH-004, REQ-HEALTH-006, REQ-HEALTH-008, NFR-SEC-003, NFR-SEC-005, NFR-SEC-006, NFR-SEC-007, NFR-OPS-006</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>A05</t>
+          <t>W04-2</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>관리자 · 운영 현황</t>
+          <t>생활습관 설문</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>기간 선택 → 단계별·날짜별 집계 → CSV</t>
+          <t>선택지 응답 → 조건부 건너뛰기 → 다음</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>체험 진행 현황, 날짜별 활동, 동의·삭제 현황, 서비스 상태, CSV</t>
+          <t>단계 표시(7단계), 선택형 문항, 운동 종목 선택·강도 자동 분류, 조건부 문항 건너뛰기, 이전·다음</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>REQ-ADM-014</t>
+          <t>REQ-HEALTH-005, REQ-PRED-008, REQ-CHAL-001, REQ-CHAL-008</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>W01</t>
+          <t>W05</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>서비스 소개 · 시작하기</t>
+          <t>입력 검토 · 분석 대기</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>소개 → 시작하기</t>
+          <t>확인 → 비동기 분석</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>서비스 한 줄 소개, 핵심 기능 3단계 안내, 시작하기 CTA</t>
+          <t>입력값 검토 요약, 분석 요청 버튼, 대기·실행·완료·실패·재시도 상태</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>REQ-HEALTH-007, REQ-PRED-002, NFR-ASYNC-001</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>W02</t>
+          <t>W06</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>회원가입 · 로그인 · 동의</t>
+          <t>예측 결과 · XAI 설명</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>계정 생성 → 필수 동의</t>
+          <t>선별 결과 → 설명 → 다음 행동</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>가입 폼, 로그인 폼, 비밀번호 재설정, 약관·건강정보 동의 체크</t>
+          <t>입력 혈압 판정, 심장 혈관 건강 신호(확률·범주·확률 근거), 혈관 나이(같은 성별·연령대 상위 %·계산 근거), 바꿀 수 있는 요인, 생활습관·체형 비교(3단계·비교 기준), 면책 문구</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>REQ-USER-001, REQ-USER-002, REQ-USER-004, REQ-CONSENT-001, REQ-CONSENT-003, NFR-SEC-003, NFR-SEC-006</t>
+          <t>REQ-PRED-001, REQ-PRED-003, REQ-PRED-006,  NFR-SAFE-001, NFR-SAFE-002, NFR-SAFE-003, NFR-SAFE-005, NFR-SAFE-007</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>W03</t>
+          <t>W07</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>이용 적합성 · 응급 확인</t>
+          <t>검사 · 상담 안내</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>안전 문진 → 서비스 분기</t>
+          <t>모델 A 높음 또는 혈압 140/90 이상 → 의료기관</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>긴급 증상 문진, 119 전화 버튼, 연령·기진단 확인, 부적합 사유 안내</t>
+          <t>고위험 안내 문구, 검사 권고, 의료기관 정보, 면책 문구</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>REQ-ELIG-001, REQ-ELIG-002, REQ-ELIG-003, REQ-ELIG-004, NFR-SAFE-004</t>
+          <t>REQ-PRED-005, NFR-SAFE-001</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>W04</t>
+          <t>W08</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>건강정보 입력</t>
+          <t>대시보드 (홈)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>직접 입력 → 검증</t>
+          <t>상태 요약 → 오늘의 실천</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>기본 정보, 계측·혈압, 가족력, 검진 결과지 사진 채우기, 필드 오류 표시, 검진 이력 추가</t>
+          <t>상단 네비게이션, 최신 위험도 카드, 오늘의 챌린지 진행률, 사이클 현황, 빈 상태 CTA</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>REQ-HEALTH-001, REQ-HEALTH-002, REQ-HEALTH-003, REQ-HEALTH-004, REQ-HEALTH-006, REQ-HEALTH-008, NFR-SEC-003, NFR-SEC-005, NFR-SEC-006, NFR-SEC-007, NFR-OPS-006</t>
+          <t>REQ-PRED-004, REQ-PRED-007, REQ-DASH-001, REQ-DASH-004, REQ-DASH-005, REQ-DASH-006, REQ-DASH-007, REQ-DASH-008, REQ-DASH-009, REQ-DASH-010, REQ-DASH-011, NFR-DASH-001, NFR-SAFE-001, NFR-SAFE-005</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>W04-2</t>
+          <t>W08-2</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>생활습관 설문</t>
+          <t>캘린더 상세</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>선택지 응답 → 조건부 건너뛰기 → 다음</t>
+          <t>날짜 선택 → 일기·사진·일정·할 일</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>단계 표시(7단계), 선택형 문항, 운동 종목 선택·강도 자동 분류, 조건부 문항 건너뛰기, 이전·다음</t>
+          <t>월 달력, 일기, 사진, 일정, 오늘 할 일(챌린지 연동)</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>REQ-HEALTH-005, REQ-PRED-008, REQ-CHAL-001, REQ-CHAL-008</t>
+          <t>REQ-CAL-001, REQ-CAL-002, REQ-CAL-003</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>W05</t>
+          <t>W09</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>입력 검토 · 분석 대기</t>
+          <t>챌린지 선택</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>확인 → 비동기 분석</t>
+          <t>추천 → 선택 → 시작</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>입력값 검토 요약, 분석 요청 버튼, 대기·실행·완료·실패·재시도 상태</t>
+          <t>예측 근거별 챌린지 후보, 연결된 위험 요인 표시, 목표 횟수 설정, 사이클 시작, 고정 미션 2개, 제외한 챌린지·이유</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>REQ-HEALTH-007, REQ-PRED-002, NFR-ASYNC-001</t>
+          <t>REQ-CHAL-001, REQ-CHAL-002, REQ-CHAL-003, REQ-CHAL-008, REQ-CHAL-009, NFR-DASH-001, REQ-FEED-003, NFR-SAFE-007</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>W06</t>
+          <t>W10</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>예측 결과 · XAI 설명</t>
+          <t>챌린지 수행 · 인증</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>선별 결과 → 설명 → 다음 행동</t>
+          <t>목표 → 인증 → 달성률</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>입력 혈압 판정, 심장 혈관 건강 신호(확률·범주·확률 근거), 혈관 나이(같은 성별·연령대 상위 %·계산 근거), 바꿀 수 있는 요인, 생활습관·체형 비교(3단계·비교 기준), 면책 문구</t>
+          <t>오늘의 목표 목록, 인증하기, 당일 기록 수정, 주간·사이클 달성률, 식단 사진 업로드</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>REQ-PRED-001, REQ-PRED-003, REQ-PRED-006,  NFR-SAFE-001, NFR-SAFE-002, NFR-SAFE-003, NFR-SAFE-005, NFR-SAFE-007</t>
+          <t>REQ-CHAL-004, REQ-CHAL-005, REQ-CHAL-006, REQ-CHAL-007, REQ-CHAL-010, REQ-DASH-008, REQ-DASH-009, NFR-DASH-001, REQ-RECO-002</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>W07</t>
+          <t>W11</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>검사 · 상담 안내</t>
+          <t>추이 · 변화 추적</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>모델 A 높음 또는 혈압 140/90 이상 → 의료기관</t>
+          <t>이력 → 차트</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>고위험 안내 문구, 검사 권고, 의료기관 정보, 면책 문구</t>
+          <t>예측 이력 차트, 최초 대비 증감(색상+기호), 기간 필터, 데이터 1건 이하 빈 상태</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>REQ-PRED-005, NFR-SAFE-001</t>
+          <t>REQ-DASH-002, REQ-DASH-003, REQ-DASH-010, REQ-FEED-002, NFR-SAFE-005, NFR-ARCH-004</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>W08</t>
+          <t>W11-2</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>대시보드 (홈)</t>
+          <t>4주 전 · 후 비교</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>상태 요약 → 오늘의 실천</t>
+          <t>재입력 → 같은 모델 → 변화</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>상단 네비게이션, 최신 위험도 카드, 오늘의 챌린지 진행률, 사이클 현황, 빈 상태 CTA</t>
+          <t>시작·4주 후 심장 혈관 건강 신호·생활습관·체형 비교, 혈압·몸무게·허리둘레 변화, 미션 달성률·습관 변화, 다음 4주 챌린지 선택 (혈관 나이·요인 순위 변화는 보류 · 결정 필요 시트 참고)</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>REQ-PRED-004, REQ-PRED-007, REQ-DASH-001, REQ-DASH-004, REQ-DASH-005, REQ-DASH-006, REQ-DASH-007, REQ-DASH-008, REQ-DASH-009, REQ-DASH-010, REQ-DASH-011, NFR-DASH-001, NFR-SAFE-001, NFR-SAFE-005</t>
+          <t>REQ-HEALTH-008, REQ-PRED-007, REQ-DASH-003, REQ-DASH-011</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>W08-2</t>
+          <t>W12</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>캘린더 상세</t>
+          <t>피드백 · 마이페이지</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>날짜 선택 → 일기·사진·일정·할 일</t>
+          <t>의견 → 저장 / 계정 관리</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>월 달력, 일기, 사진, 일정, 오늘 할 일(챌린지 연동)</t>
+          <t>결과·추천 평가와 의견 입력, 알림 수신 설정, 동의 철회, 회원 탈퇴</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>REQ-CAL-001, REQ-CAL-002, REQ-CAL-003</t>
+          <t>REQ-USER-003, REQ-CONSENT-002, REQ-NOTI-001, REQ-FEED-001</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>W09</t>
+          <t>W13</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>챌린지 선택</t>
+          <t>커뮤니티 피드</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>추천 → 선택 → 시작</t>
+          <t>피드 보기 → 글 열기 / 글쓰기 / 사람 프로필</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>예측 근거별 챌린지 후보, 연결된 위험 요인 표시, 목표 횟수 설정, 사이클 시작, 고정 미션 2개, 제외한 챌린지·이유</t>
+          <t>탭(피드·챌린지·파티), 분류 칩, 안내 띠, 글 카드, 글쓰기 버튼</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>REQ-CHAL-001, REQ-CHAL-002, REQ-CHAL-003, REQ-CHAL-008, REQ-CHAL-009, NFR-DASH-001, REQ-FEED-003, NFR-SAFE-007</t>
+          <t>REQ-COMM-001, REQ-COMM-002, REQ-COMM-003, REQ-COMM-007, REQ-COMM-010, REQ-PUSH-001</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W14</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>챌린지 수행 · 인증</t>
+          <t>글쓰기</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>목표 → 인증 → 달성률</t>
+          <t>분류 선택 → 제목·본문 → 챌린지 붙이기 → 올리기</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>오늘의 목표 목록, 인증하기, 당일 기록 수정, 주간·사이클 달성률, 식단 사진 업로드</t>
+          <t>올릴 곳, 분류 칩, 제목·본문, 챌린지 붙이기, 사진 3장, 파이 안내</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>REQ-CHAL-004, REQ-CHAL-005, REQ-CHAL-006, REQ-CHAL-007, REQ-CHAL-010, REQ-DASH-008, REQ-DASH-009, NFR-DASH-001, REQ-RECO-002</t>
+          <t>REQ-COMM-004, REQ-COMM-005, REQ-COMM-007, REQ-PIE-001</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W15</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>추이 · 변화 추적</t>
+          <t>글 상세 · 댓글 · 답글 · 좋아요</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>이력 → 차트</t>
+          <t>글 읽기 → 좋아요 → 댓글·답글 → 수정·삭제·신고</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>예측 이력 차트, 최초 대비 증감(색상+기호), 기간 필터, 데이터 1건 이하 빈 상태</t>
+          <t>글 머리, 좋아요, 신고, 댓글·답글(한 단계), 댓글 좋아요, 입력줄</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>REQ-DASH-002, REQ-DASH-003, REQ-DASH-010, REQ-FEED-002, NFR-SAFE-005, NFR-ARCH-004</t>
+          <t>REQ-COMM-003, REQ-COMM-005, REQ-COMM-006, REQ-COMM-008, REQ-COMM-009, REQ-COMM-010, REQ-PUSH-002</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>W11-2</t>
+          <t>W16</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>4주 전 · 후 비교</t>
+          <t>사람 프로필 · 인기도</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>재입력 → 같은 모델 → 변화</t>
+          <t>닉네임·아바타 → 글·댓글 → 인기도 하트</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>시작·4주 후 심장 혈관 건강 신호·생활습관·체형 비교, 혈압·몸무게·허리둘레 변화, 미션 달성률·습관 변화, 다음 4주 챌린지 선택 (혈관 나이·요인 순위 변화는 보류 · 결정 필요 시트 참고)</t>
+          <t>캐릭터·닉네임, 인기도 하트, 글·댓글 탭</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>REQ-HEALTH-008, REQ-PRED-007, REQ-DASH-003, REQ-DASH-011</t>
+          <t>REQ-COMM-011, REQ-COMM-012, REQ-COMM-013, REQ-CHARA-003, REQ-PUSH-005</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W17</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>피드백 · 마이페이지</t>
+          <t>닉네임 정하기 · 캐릭터 꾸미기</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>의견 → 저장 / 계정 관리</t>
+          <t>닉네임 → 캐릭터 → 파이로 아이템 구매 → 저장</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>결과·추천 평가와 의견 입력, 알림 수신 설정, 동의 철회, 회원 탈퇴</t>
+          <t>미리보기, 6개 탭(몸체·색·눈 색·표정·얼굴·머리), 가격, 파이 잔액, 저장 버튼</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>REQ-USER-003, REQ-CONSENT-002, REQ-NOTI-001, REQ-FEED-001</t>
+          <t>REQ-COMM-014, REQ-CHARA-001, REQ-CHARA-002, REQ-CHARA-003, REQ-PIE-002</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>W13</t>
+          <t>W18</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>커뮤니티 피드</t>
+          <t>파이</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>피드 보기 → 글 열기 / 글쓰기 / 사람 프로필</t>
+          <t>내 파이 → 모으는 방법 → 최근 내역</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>탭(피드·챌린지·파티), 분류 칩, 안내 띠, 글 카드, 글쓰기 버튼</t>
+          <t>잔액, 지급표, 최근 내역, 가입 감사 파이 받기</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>REQ-COMM-001, REQ-COMM-002, REQ-COMM-003, REQ-COMM-007, REQ-COMM-010, REQ-PUSH-001</t>
+          <t>REQ-PIE-001, REQ-PIE-002, REQ-PIE-003, REQ-PIE-004</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W19</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>글쓰기</t>
+          <t>챌린지 파티</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>분류 선택 → 제목·본문 → 챌린지 붙이기 → 올리기</t>
+          <t>만들기 / 초대 코드 참여 → 파티 현황 → 파티 피드</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>올릴 곳, 분류 칩, 제목·본문, 챌린지 붙이기, 사진 3장, 파이 안내</t>
+          <t>파티 시작·만들기·현황·피드(W19-2~4 하위 화면)</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>REQ-COMM-004, REQ-COMM-005, REQ-COMM-007, REQ-PIE-001</t>
+          <t>REQ-PARTY-001, REQ-PARTY-002, REQ-PARTY-003, REQ-PARTY-004, REQ-PARTY-005, REQ-PUSH-004</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>W15</t>
+          <t>W20</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>글 상세 · 댓글 · 답글 · 좋아요</t>
+          <t>공통 챌린지</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>글 읽기 → 좋아요 → 댓글·답글 → 수정·삭제·신고</t>
+          <t>목록 → 참여 → 하루 인증 → 순위·완주 보상</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>글 머리, 좋아요, 신고, 댓글·답글(한 단계), 댓글 좋아요, 입력줄</t>
+          <t>목록(진행·예정·종료), 상세(규칙·보상·순위표), 인증 입력</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>REQ-COMM-003, REQ-COMM-005, REQ-COMM-006, REQ-COMM-008, REQ-COMM-009, REQ-COMM-010, REQ-PUSH-002</t>
+          <t>REQ-CCHAL-001, REQ-CCHAL-002, REQ-CCHAL-003, REQ-CCHAL-004, REQ-CCHAL-005</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>W16</t>
+          <t>W21</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>사람 프로필 · 인기도</t>
+          <t>1:1 문의 · 비회원 문의 · 공지사항</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>닉네임·아바타 → 글·댓글 → 인기도 하트</t>
+          <t>문의 남기기 → 답변 확인 / 공지 확인</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>캐릭터·닉네임, 인기도 하트, 글·댓글 탭</t>
+          <t>문의 목록·작성, 비회원 문의(조회 번호), 공지 목록</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>REQ-COMM-011, REQ-COMM-012, REQ-COMM-013, REQ-CHARA-003, REQ-PUSH-005</t>
+          <t>REQ-INQ-001, REQ-INQ-002, REQ-INQ-003, REQ-INQ-004, REQ-NOTICE-002, REQ-PUSH-003</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>W22</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>닉네임 정하기 · 캐릭터 꾸미기</t>
+          <t>알림 설정 · 더보기</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>닉네임 → 캐릭터 → 파이로 아이템 구매 → 저장</t>
+          <t>더보기 → 알림 설정 → 켜기 → 종류별 선택</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>미리보기, 6개 탭(몸체·색·눈 색·표정·얼굴·머리), 가격, 파이 잔액, 저장 버튼</t>
+          <t>알림 스위치, 종류별 스위치 5개, 환경 안내(아이폰·안드로이드), 더보기 메뉴</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>REQ-COMM-014, REQ-CHARA-001, REQ-CHARA-002, REQ-CHARA-003, REQ-PIE-002</t>
+          <t>REQ-PUSH-001, REQ-PUSH-002, REQ-PUSH-003, REQ-PUSH-004, REQ-PUSH-005, REQ-PUSH-006, REQ-PUSH-007, REQ-NOTI-001</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>W18</t>
+          <t>W23</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>파이</t>
+          <t>내 12주 계획 · 12주 결과 · 지난 12주 기록</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>내 파이 → 모으는 방법 → 최근 내역</t>
+          <t>12주 계획 → 4주마다 재입력 → 12주 결과 → 지난 기록</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>잔액, 지급표, 최근 내역, 가입 감사 파이 받기</t>
+          <t>12주 일정, 혈압 그래프, 전·후 표, 습관 변화, 4주마다 달성률</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>REQ-PIE-001, REQ-PIE-002, REQ-PIE-003, REQ-PIE-004</t>
+          <t>REQ-CHAL-012, REQ-CHAL-013, REQ-DASH-012, REQ-DASH-013, NFR-SAFE-001</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>W19</t>
+          <t>W24</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>챌린지 파티</t>
+          <t>내 배지</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>만들기 / 초대 코드 참여 → 파티 현황 → 파티 피드</t>
+          <t>배지 모으기 → 내 배지 확인</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>파티 시작·만들기·현황·피드(W19-2~4 하위 화면)</t>
+          <t>모은 개수 링, 다음 배지, 연속 달성·완주와 기록 배지, 진행률</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>REQ-PARTY-001, REQ-PARTY-002, REQ-PARTY-003, REQ-PARTY-004, REQ-PARTY-005, REQ-PUSH-004</t>
+          <t>REQ-BADGE-001, REQ-BADGE-002</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>W20</t>
+          <t>A01</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>공통 챌린지</t>
+          <t>관리자 · 미션 · 가입자 · 통계 · 열람 기록</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>목록 → 참여 → 하루 인증 → 순위·완주 보상</t>
+          <t>미션 노출 → 가입자 → 통계 → 열람 기록</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>목록(진행·예정·종료), 상세(규칙·보상·순위표), 인증 입력</t>
+          <t>왼쪽 메뉴(11개), 표, 필터, 검색</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>REQ-CCHAL-001, REQ-CCHAL-002, REQ-CCHAL-003, REQ-CCHAL-004, REQ-CCHAL-005</t>
+          <t>REQ-ADM-001, REQ-ADM-002, REQ-ADM-003, REQ-ADM-004, REQ-ADM-012</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>W21</t>
+          <t>A02</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>1:1 문의 · 비회원 문의 · 공지사항</t>
+          <t>관리자 · 문의 · 비회원 문의</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>문의 남기기 → 답변 확인 / 공지 확인</t>
+          <t>목록 → 열어서 답변</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>문의 목록·작성, 비회원 문의(조회 번호), 공지 목록</t>
+          <t>상태 필터, 문의 목록, 답변 입력</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>REQ-INQ-001, REQ-INQ-002, REQ-INQ-003, REQ-INQ-004, REQ-NOTICE-002, REQ-PUSH-003</t>
+          <t>REQ-ADM-005, REQ-ADM-006, REQ-INQ-002, REQ-INQ-003</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>W22</t>
+          <t>A03</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>알림 설정 · 더보기</t>
+          <t>관리자 · 공지 · 신고 · 글 관리</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>더보기 → 알림 설정 → 켜기 → 종류별 선택</t>
+          <t>공지 올리기 / 신고 처리 / 글 숨김·삭제</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>알림 스위치, 종류별 스위치 5개, 환경 안내(아이폰·안드로이드), 더보기 메뉴</t>
+          <t>공지 폼, 신고 표, 글 표, 계정 정지·삭제</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>REQ-PUSH-001, REQ-PUSH-002, REQ-PUSH-003, REQ-PUSH-004, REQ-PUSH-005, REQ-PUSH-006, REQ-PUSH-007, REQ-NOTI-001</t>
+          <t>REQ-ADM-007, REQ-ADM-008, REQ-ADM-009, REQ-ADM-013, REQ-NOTICE-001, REQ-COMM-008</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>W23</t>
+          <t>A04</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>내 12주 계획 · 12주 결과 · 지난 12주 기록</t>
+          <t>관리자 · 공통 챌린지 · 테스트 계정 삭제</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>12주 계획 → 4주마다 재입력 → 12주 결과 → 지난 기록</t>
+          <t>공통 챌린지 열기·확정 / 테스트 계정 삭제</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>12주 일정, 혈압 그래프, 전·후 표, 습관 변화, 4주마다 달성률</t>
+          <t>챌린지 폼·카드, 순위 확정, 미리보기·삭제</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>REQ-CHAL-012, REQ-CHAL-013, REQ-DASH-012, REQ-DASH-013, NFR-SAFE-001</t>
+          <t>REQ-ADM-010, REQ-ADM-011, REQ-CCHAL-005</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>W24</t>
+          <t>A05</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>내 배지</t>
+          <t>관리자 · 운영 현황</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>배지 모으기 → 내 배지 확인</t>
+          <t>기간 선택 → 단계별·날짜별 집계 → CSV</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>모은 개수 링, 다음 배지, 연속 달성·완주와 기록 배지, 진행률</t>
+          <t>체험 진행 현황, 날짜별 활동, 동의·삭제 현황, 서비스 상태, CSV</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>REQ-BADGE-001, REQ-BADGE-002</t>
+          <t>REQ-ADM-014</t>
         </is>
       </c>
     </row>

</xml_diff>